<commit_message>
Update: Before the last edition
</commit_message>
<xml_diff>
--- a/output/step1/meta/Data_D_10_manifest.xlsx
+++ b/output/step1/meta/Data_D_10_manifest.xlsx
@@ -611,7 +611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -634,7 +634,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Raw_Data/Raw_Data_Daily.xlsx</t>
+          <t>../raw_data/Raw_Data_Daily.xlsx</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Raw_Data/Raw_Data_Monthly+.xlsx</t>
+          <t>../raw_data/Raw_Data_Monthly+.xlsx</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>../output/step1</t>
         </is>
       </c>
     </row>
@@ -743,110 +743,120 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>FEATURES.tech_windows_days</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>[5, 20, 60]</t>
-        </is>
+          <t>RUN.enforce_label_availability</t>
+        </is>
+      </c>
+      <c r="B12" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FEATURES.lags_days</t>
+          <t>FEATURES.tech_windows_days</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>[1, 2, 5, 10, 20]</t>
+          <t>[5, 20, 60]</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PLOTS.font_family_candidates</t>
+          <t>FEATURES.lags_days</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>['Microsoft YaHei', 'SimHei', 'PingFang SC', 'Noto Sans CJK SC', 'Arial Unicode MS']</t>
+          <t>[1, 2, 5, 10, 20]</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PLOTS.base_font_size</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>11</v>
+          <t>PLOTS.font_family_candidates</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>['Microsoft YaHei', 'SimHei', 'SimSun', 'Arial']</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PLOTS.dpi</t>
+          <t>PLOTS.base_font_size</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>220</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PLOTS.plot2_vars</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>['VIX', 'US_TermSpread', 'WTI', 'GOLD', 'EPU_D']</t>
-        </is>
+          <t>PLOTS.dpi</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>220</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PLOTS.plot3_vars</t>
+          <t>PLOTS.plot2_vars</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>['USD_1', 'VIX', 'US_TermSpread', 'WTI', 'GOLD', 'EPU_D', 'USD_EUR', 'USD_JPY', 'USD_GBP', 'USD_CNY']</t>
+          <t>['VIX', 'US_TermSpread', 'WTI', 'GOLD', 'EPU_D']</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PLOTS.plot4_top_n</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>30</v>
+          <t>PLOTS.plot3_vars</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>['USD_1', 'VIX', 'US_TermSpread', 'WTI', 'GOLD', 'EPU_D', 'USD_EUR', 'USD_JPY', 'USD_GBP', 'USD_CNY']</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>LOWFREQ_LAG.monthly</t>
+          <t>PLOTS.plot4_top_n</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>LOWFREQ_LAG.monthly</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>LOWFREQ_LAG.quarterly</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="B22" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update: The Final Edition
</commit_message>
<xml_diff>
--- a/output/step1/meta/Data_D_10_manifest.xlsx
+++ b/output/step1/meta/Data_D_10_manifest.xlsx
@@ -460,7 +460,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>表1_变量清单与处理口径.xlsx</t>
+          <t>表1_变量清单与处理口径_H10.xlsx</t>
         </is>
       </c>
     </row>
@@ -477,7 +477,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>表2_缺失率与样本覆盖.xlsx</t>
+          <t>表2_缺失率与样本覆盖_H10.xlsx</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>表3_描述统计.xlsx</t>
+          <t>表3_描述统计_H10.xlsx</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>表4_样本筛选统计.xlsx</t>
+          <t>表4_样本筛选统计_H10.xlsx</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>图1_USD持有期对数收益标签时间序列.png</t>
+          <t>图1_USD持有期对数收益标签时间序列_H10.png</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>图2_关键外生变量时间序列.png</t>
+          <t>图2_关键外生变量时间序列_H10.png</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>图3_相关性热力图.png</t>
+          <t>图3_相关性热力图_H10.png</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>图4_缺失分布可视化.png</t>
+          <t>图4_缺失分布可视化_H10.png</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>图5_低频滞后与日度映射示意图.png</t>
+          <t>图5_低频滞后与日度映射示意图_H10.png</t>
         </is>
       </c>
     </row>

</xml_diff>